<commit_message>
Adding the column time
</commit_message>
<xml_diff>
--- a/rag/excel/matrix_cohen.xlsx
+++ b/rag/excel/matrix_cohen.xlsx
@@ -1369,7 +1369,6 @@
       <c r="J11" t="n">
         <v>31</v>
       </c>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
         <v>0.7519998311488212</v>
       </c>
@@ -1458,7 +1457,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -1473,16 +1472,16 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="L2" t="n">
-        <v>0.5636505211037015</v>
+        <v>0.6898891937747429</v>
       </c>
     </row>
     <row r="3">
@@ -1495,7 +1494,7 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -1519,10 +1518,10 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="L3" t="n">
-        <v>0.5636505211037015</v>
+        <v>0.6898891937747429</v>
       </c>
     </row>
     <row r="4">
@@ -1532,13 +1531,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -1559,10 +1558,10 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="L4" t="n">
-        <v>0.5636505211037015</v>
+        <v>0.6898891937747429</v>
       </c>
     </row>
     <row r="5">
@@ -1572,7 +1571,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -1599,10 +1598,10 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L5" t="n">
-        <v>0.5636505211037015</v>
+        <v>0.6898891937747429</v>
       </c>
     </row>
     <row r="6">
@@ -1612,10 +1611,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -1624,10 +1623,10 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -1639,10 +1638,10 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L6" t="n">
-        <v>0.5636505211037015</v>
+        <v>0.6898891937747429</v>
       </c>
     </row>
     <row r="7">
@@ -1652,7 +1651,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -1667,7 +1666,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -1676,13 +1675,13 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K7" t="n">
         <v>21</v>
       </c>
       <c r="L7" t="n">
-        <v>0.5636505211037015</v>
+        <v>0.6898891937747429</v>
       </c>
     </row>
     <row r="8">
@@ -1695,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -1707,10 +1706,10 @@
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H8" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="I8" t="n">
         <v>1</v>
@@ -1719,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="L8" t="n">
-        <v>0.5636505211037015</v>
+        <v>0.6898891937747429</v>
       </c>
     </row>
     <row r="9">
@@ -1732,37 +1731,37 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I9" t="n">
+        <v>14</v>
+      </c>
+      <c r="J9" t="n">
         <v>12</v>
       </c>
-      <c r="J9" t="n">
-        <v>11</v>
-      </c>
       <c r="K9" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="L9" t="n">
-        <v>0.5636505211037015</v>
+        <v>0.6898891937747429</v>
       </c>
     </row>
     <row r="10">
@@ -1772,7 +1771,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -1796,13 +1795,13 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K10" t="n">
         <v>23</v>
       </c>
       <c r="L10" t="n">
-        <v>0.5636505211037015</v>
+        <v>0.6898891937747429</v>
       </c>
     </row>
     <row r="11">
@@ -1812,34 +1811,35 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="C11" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D11" t="n">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G11" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H11" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="I11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J11" t="n">
-        <v>32</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>0.5636505211037015</v>
+        <v>0.6898891937747429</v>
       </c>
     </row>
   </sheetData>
@@ -1926,7 +1926,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -1938,7 +1938,7 @@
         <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
         <v>1</v>
@@ -1950,7 +1950,7 @@
         <v>23</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7128168390889362</v>
+        <v>0.7230872822153017</v>
       </c>
     </row>
     <row r="3">
@@ -1960,10 +1960,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -1990,7 +1990,7 @@
         <v>26</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7128168390889362</v>
+        <v>0.7230872822153017</v>
       </c>
     </row>
     <row r="4">
@@ -2000,13 +2000,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -2030,7 +2030,7 @@
         <v>51</v>
       </c>
       <c r="L4" t="n">
-        <v>0.7128168390889362</v>
+        <v>0.7230872822153017</v>
       </c>
     </row>
     <row r="5">
@@ -2070,7 +2070,7 @@
         <v>3</v>
       </c>
       <c r="L5" t="n">
-        <v>0.7128168390889362</v>
+        <v>0.7230872822153017</v>
       </c>
     </row>
     <row r="6">
@@ -2080,10 +2080,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -2092,25 +2092,25 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="n">
         <v>8</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7128168390889362</v>
+        <v>0.7230872822153017</v>
       </c>
     </row>
     <row r="7">
@@ -2123,7 +2123,7 @@
         <v>5</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H7" t="n">
         <v>1</v>
@@ -2150,7 +2150,7 @@
         <v>21</v>
       </c>
       <c r="L7" t="n">
-        <v>0.7128168390889362</v>
+        <v>0.7230872822153017</v>
       </c>
     </row>
     <row r="8">
@@ -2166,7 +2166,7 @@
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -2175,10 +2175,10 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -2190,7 +2190,7 @@
         <v>34</v>
       </c>
       <c r="L8" t="n">
-        <v>0.7128168390889362</v>
+        <v>0.7230872822153017</v>
       </c>
     </row>
     <row r="9">
@@ -2200,37 +2200,37 @@
         </is>
       </c>
       <c r="B9" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
         <v>9</v>
       </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>11</v>
-      </c>
       <c r="I9" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K9" t="n">
         <v>46</v>
       </c>
       <c r="L9" t="n">
-        <v>0.7128168390889362</v>
+        <v>0.7230872822153017</v>
       </c>
     </row>
     <row r="10">
@@ -2258,19 +2258,19 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I10" t="n">
         <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K10" t="n">
         <v>23</v>
       </c>
       <c r="L10" t="n">
-        <v>0.7128168390889362</v>
+        <v>0.7230872822153017</v>
       </c>
     </row>
     <row r="11">
@@ -2280,34 +2280,34 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C11" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D11" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G11" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H11" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="I11" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J11" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="L11" t="n">
-        <v>0.7128168390889362</v>
+        <v>0.7230872822153017</v>
       </c>
     </row>
   </sheetData>
@@ -2856,7 +2856,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
@@ -2883,10 +2883,10 @@
         <v>1</v>
       </c>
       <c r="K2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6367390153520383</v>
+        <v>0.6159804753820034</v>
       </c>
     </row>
     <row r="3">
@@ -2902,7 +2902,7 @@
         <v>23</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -2917,7 +2917,7 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -2926,7 +2926,7 @@
         <v>26</v>
       </c>
       <c r="L3" t="n">
-        <v>0.6367390153520383</v>
+        <v>0.6159804753820034</v>
       </c>
     </row>
     <row r="4">
@@ -2936,13 +2936,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -2957,7 +2957,7 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -2966,7 +2966,7 @@
         <v>51</v>
       </c>
       <c r="L4" t="n">
-        <v>0.6367390153520383</v>
+        <v>0.6159804753820034</v>
       </c>
     </row>
     <row r="5">
@@ -3006,7 +3006,7 @@
         <v>3</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6367390153520383</v>
+        <v>0.6159804753820034</v>
       </c>
     </row>
     <row r="6">
@@ -3016,13 +3016,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -3031,13 +3031,13 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -3046,7 +3046,7 @@
         <v>8</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6367390153520383</v>
+        <v>0.6159804753820034</v>
       </c>
     </row>
     <row r="7">
@@ -3056,7 +3056,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -3068,10 +3068,10 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H7" t="n">
         <v>1</v>
@@ -3086,7 +3086,7 @@
         <v>21</v>
       </c>
       <c r="L7" t="n">
-        <v>0.6367390153520383</v>
+        <v>0.6159804753820034</v>
       </c>
     </row>
     <row r="8">
@@ -3099,10 +3099,10 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -3114,10 +3114,10 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -3126,7 +3126,7 @@
         <v>32</v>
       </c>
       <c r="L8" t="n">
-        <v>0.6367390153520383</v>
+        <v>0.6159804753820034</v>
       </c>
     </row>
     <row r="9">
@@ -3136,7 +3136,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -3148,25 +3148,25 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="I9" t="n">
         <v>29</v>
       </c>
       <c r="J9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
         <v>46</v>
       </c>
       <c r="L9" t="n">
-        <v>0.6367390153520383</v>
+        <v>0.6159804753820034</v>
       </c>
     </row>
     <row r="10">
@@ -3179,16 +3179,16 @@
         <v>5</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -3197,16 +3197,16 @@
         <v>4</v>
       </c>
       <c r="I10" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" t="n">
         <v>4</v>
       </c>
-      <c r="J10" t="n">
-        <v>5</v>
-      </c>
       <c r="K10" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L10" t="n">
-        <v>0.6367390153520383</v>
+        <v>0.6159804753820034</v>
       </c>
     </row>
     <row r="11">
@@ -3216,13 +3216,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D11" t="n">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
@@ -3231,19 +3231,19 @@
         <v>2</v>
       </c>
       <c r="G11" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H11" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I11" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L11" t="n">
-        <v>0.6367390153520383</v>
+        <v>0.6159804753820034</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
try to grasp energy with worker
</commit_message>
<xml_diff>
--- a/rag/excel/matrix_cohen.xlsx
+++ b/rag/excel/matrix_cohen.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="mistral_Rag" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="phi4_Rag" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="llama3.3_Rag" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -506,13 +508,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -527,16 +529,16 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="L2" t="n">
-        <v>0.01269444595353217</v>
+        <v>0.6007051377354883</v>
       </c>
     </row>
     <row r="3">
@@ -546,13 +548,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -573,10 +575,10 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="L3" t="n">
-        <v>0.01269444595353217</v>
+        <v>0.6007051377354883</v>
       </c>
     </row>
     <row r="4">
@@ -586,13 +588,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -613,10 +615,10 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="L4" t="n">
-        <v>0.01269444595353217</v>
+        <v>0.6007051377354883</v>
       </c>
     </row>
     <row r="5">
@@ -626,7 +628,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -635,7 +637,7 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -653,10 +655,10 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L5" t="n">
-        <v>0.01269444595353217</v>
+        <v>0.6007051377354883</v>
       </c>
     </row>
     <row r="6">
@@ -666,13 +668,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -684,19 +686,19 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L6" t="n">
-        <v>0.01269444595353217</v>
+        <v>0.6007051377354883</v>
       </c>
     </row>
     <row r="7">
@@ -706,7 +708,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -721,22 +723,22 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="L7" t="n">
-        <v>0.01269444595353217</v>
+        <v>0.6007051377354883</v>
       </c>
     </row>
     <row r="8">
@@ -749,10 +751,10 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -761,10 +763,10 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -773,10 +775,10 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="L8" t="n">
-        <v>0.01269444595353217</v>
+        <v>0.6007051377354883</v>
       </c>
     </row>
     <row r="9">
@@ -786,7 +788,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -801,22 +803,22 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="L9" t="n">
-        <v>0.01269444595353217</v>
+        <v>0.6007051377354883</v>
       </c>
     </row>
     <row r="10">
@@ -826,13 +828,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -844,19 +846,19 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="L10" t="n">
-        <v>0.01269444595353217</v>
+        <v>0.6007051377354883</v>
       </c>
     </row>
     <row r="11">
@@ -866,35 +868,971 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.6007051377354883</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SumRow</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>22</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.6996710733066561</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>26</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>26</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.6996710733066561</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>49</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>51</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.6996710733066561</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.6996710733066561</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.6996710733066561</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>17</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>21</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.6996710733066561</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>29</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>34</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.6996710733066561</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" t="n">
+        <v>8</v>
+      </c>
+      <c r="I9" t="n">
+        <v>12</v>
+      </c>
+      <c r="J9" t="n">
+        <v>15</v>
+      </c>
+      <c r="K9" t="n">
+        <v>46</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.6996710733066561</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>21</v>
+      </c>
+      <c r="K10" t="n">
+        <v>23</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.6996710733066561</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>SumCol</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>27</v>
+      </c>
+      <c r="C11" t="n">
+        <v>28</v>
+      </c>
+      <c r="D11" t="n">
+        <v>55</v>
+      </c>
+      <c r="E11" t="n">
+        <v>6</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>24</v>
+      </c>
+      <c r="H11" t="n">
+        <v>39</v>
+      </c>
+      <c r="I11" t="n">
+        <v>13</v>
+      </c>
+      <c r="J11" t="n">
+        <v>39</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.6996710733066561</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SumRow</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Interpret</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" t="n">
+        <v>23</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.727521872035417</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.RF</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>26</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>26</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.727521872035417</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>MonCal.Facts.DC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>49</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>51</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.727521872035417</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>BDS.Emotions</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.727521872035417</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.Value</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.727521872035417</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>MotOrient.SelfEff</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>14</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>21</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.727521872035417</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>DomKldg</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>31</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>34</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.727521872035417</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>StratKldg</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>10</v>
+      </c>
+      <c r="I9" t="n">
+        <v>18</v>
+      </c>
+      <c r="J9" t="n">
+        <v>8</v>
+      </c>
+      <c r="K9" t="n">
+        <v>46</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.727521872035417</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>CTRL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>20</v>
+      </c>
+      <c r="K10" t="n">
+        <v>23</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.727521872035417</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>SumCol</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>33</v>
+      </c>
+      <c r="C11" t="n">
+        <v>27</v>
+      </c>
+      <c r="D11" t="n">
+        <v>52</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>18</v>
+      </c>
+      <c r="H11" t="n">
+        <v>46</v>
+      </c>
+      <c r="I11" t="n">
+        <v>21</v>
+      </c>
+      <c r="J11" t="n">
+        <v>32</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>0.01269444595353217</v>
+        <v>0.727521872035417</v>
       </c>
     </row>
   </sheetData>

</xml_diff>